<commit_message>
add metrics in automatic prevention
</commit_message>
<xml_diff>
--- a/dataset/Automatic-Prevention.xlsx
+++ b/dataset/Automatic-Prevention.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Desktop\cisb++\literature review\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F022FD2-DFB7-49C7-AC0F-8903DA07EF2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{267AD15E-B2D6-49B9-9B29-22BC998C4A0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5625" yWindow="2970" windowWidth="31950" windowHeight="16920" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6090" yWindow="3900" windowWidth="31950" windowHeight="16920" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="new CISB" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="84">
   <si>
     <t>Prevention</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -121,9 +121,6 @@
     <t>Binsec/rel: symbolic binary analyzer for security with applications to constant-time and secret-erasure</t>
   </si>
   <si>
-    <t>Optimization-directed compiler fuzzing for continuous translation validation</t>
-  </si>
-  <si>
     <t>Do you even lift? Strengthening compiler security guarantees against spectre attacks</t>
   </si>
   <si>
@@ -170,10 +167,6 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>优化导向的 translation validation</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>防御攻击面：Spectre</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
@@ -206,14 +199,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>一种优化导向的 fuzzing 框架，生成特定优化的程序，利用 translation validation 验证优化正确性</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>更接近 miscopilation</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>关于常数时间和 secret-erasure 的验证方法，可用于漏洞检测。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -261,11 +246,111 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>compcert 扩展</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>设计了一种区域化 C 程序的编译器，保证形式化安全。通过机器检查和区域化隔离 UB 执行的影响。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>所有 UB</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Year</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Type</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Target</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>FP</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>FN</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PO</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DD&amp;RP</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>优化后无法被 sanitizer 检测的 bug</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Ispec 1, 2, 3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>no</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>yes</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>V</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Ispec 3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>F</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Opsec 2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Opsec 1, 2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>RP</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Opsec 3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Opsec 2, 3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>C&amp;V</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;1%</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>16.69% full 103.8%</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SD&amp;V</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Ospec 3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>user 4% kernel 32%</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -325,7 +410,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -338,6 +423,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -722,219 +816,365 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB2953D7-F2D6-42FD-AC8D-897AE28D5166}">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="39.125" style="4" customWidth="1"/>
     <col min="2" max="3" width="25.875" customWidth="1"/>
-    <col min="4" max="4" width="23" customWidth="1"/>
-    <col min="5" max="5" width="14.625" customWidth="1"/>
+    <col min="4" max="4" width="18.5" customWidth="1"/>
+    <col min="5" max="5" width="12.375" customWidth="1"/>
+    <col min="6" max="6" width="20.625" customWidth="1"/>
+    <col min="7" max="7" width="14.625" customWidth="1"/>
+    <col min="8" max="10" width="8.625" customWidth="1"/>
+    <col min="11" max="11" width="14.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="28.5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" ht="28.5" x14ac:dyDescent="0.2">
+      <c r="F1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>18</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="28.5" x14ac:dyDescent="0.2">
+        <v>30</v>
+      </c>
+      <c r="E2" s="2">
+        <v>2023</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="J2" s="5">
+        <v>0.04</v>
+      </c>
+      <c r="K2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>19</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="42.75" x14ac:dyDescent="0.2">
+        <v>30</v>
+      </c>
+      <c r="E3" s="2">
+        <v>2024</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>23</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E4" s="1">
+        <v>2025</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="H4" s="1"/>
+      <c r="I4" s="1"/>
+      <c r="J4" s="1"/>
+      <c r="K4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="42.75" x14ac:dyDescent="0.2">
+      <c r="A5" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C5" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="D4" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="E4" t="s">
+      <c r="D5" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E5" s="1">
+        <v>2023</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H5" s="1"/>
+      <c r="I5" s="1"/>
+      <c r="J5" s="1"/>
+      <c r="K5" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="57" x14ac:dyDescent="0.2">
-      <c r="A5" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="E5" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="42.75" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:11" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>49</v>
       </c>
       <c r="D6" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E6" s="1">
+        <v>2024</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+      <c r="J6" s="6">
+        <v>0.21299999999999999</v>
+      </c>
+      <c r="K6" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="28.5" x14ac:dyDescent="0.2">
+      <c r="A7" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E7" s="1">
+        <v>2025</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="H7" s="1"/>
+      <c r="I7" s="1"/>
+      <c r="J7" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="K7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="42.75" x14ac:dyDescent="0.2">
+      <c r="A8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E8" s="2">
+        <v>2022</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="H8" s="2"/>
+      <c r="I8" s="2"/>
+      <c r="J8" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="42.75" x14ac:dyDescent="0.2">
+      <c r="A9" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="E6" t="s">
+      <c r="C9" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E9" s="2">
+        <v>2025</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="H9" s="2"/>
+      <c r="I9" s="2"/>
+      <c r="J9" s="2"/>
+      <c r="K9" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="57" x14ac:dyDescent="0.2">
+      <c r="A10" s="3" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" ht="42.75" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E7" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="28.5" x14ac:dyDescent="0.2">
-      <c r="A8" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E8" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="42.75" x14ac:dyDescent="0.2">
-      <c r="A9" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C9" s="2" t="s">
+      <c r="B10" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E10" s="2">
+        <v>2025</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="H10" s="2"/>
+      <c r="I10" s="2"/>
+      <c r="J10" s="2"/>
+      <c r="K10" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="57" x14ac:dyDescent="0.2">
+      <c r="A11" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="D9" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="42.75" x14ac:dyDescent="0.2">
-      <c r="A10" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C10" s="2" t="s">
+      <c r="D11" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E11" s="2">
+        <v>2024</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="H11" s="2"/>
+      <c r="I11" s="2"/>
+      <c r="J11" s="2"/>
+      <c r="K11" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="57" x14ac:dyDescent="0.2">
-      <c r="A11" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="57" x14ac:dyDescent="0.2">
-      <c r="A12" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>61</v>
-      </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D16">
-    <sortCondition ref="D2:D16"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D15">
+    <sortCondition ref="D2:D15"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>